<commit_message>
Actualiza procesos SEACE (26/10/2026 09:35)
</commit_message>
<xml_diff>
--- a/seace/Procesos_SEACE_ATU.xlsx
+++ b/seace/Procesos_SEACE_ATU.xlsx
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E67" headerRowCount="1">
-  <autoFilter ref="A1:E67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E69" headerRowCount="1">
+  <autoFilter ref="A1:E69"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Nomenclatura"/>
     <tableColumn id="2" name="Fecha publicación"/>
@@ -617,7 +617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Convocatorias desde 2025 · Revisados: 101 · Vigentes: 15 · Generado: 23/10/2026 17:34 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
+          <t>Convocatorias desde 2025 · Revisados: 101 · Vigentes: 15 · Generado: 26/10/2026 09:35 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         <v>46317.78611111111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -797,12 +797,12 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Consultas y observaciones hasta el 27/10/2026 (4 días).</t>
+          <t>Consultas y observaciones hasta el 27/10/2026 (1 días).</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 1 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 4 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
         </is>
       </c>
       <c r="V5" s="8" t="inlineStr">
@@ -844,7 +844,7 @@
         <v>46304.93541666667</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 14 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
+          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 17 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
         </is>
       </c>
       <c r="V6" s="8" t="inlineStr">
@@ -928,7 +928,7 @@
         <v>46296.87777777778</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 22 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 25 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
         </is>
       </c>
       <c r="V7" s="8" t="inlineStr">
@@ -1006,7 +1006,7 @@
         <v>46276.85416666666</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 42 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 45 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
         </is>
       </c>
       <c r="V8" s="8" t="inlineStr">
@@ -1084,7 +1084,7 @@
         <v>46224.80069444444</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
@@ -1107,20 +1107,20 @@
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="S9" s="6" t="n">
-        <v>46224.80069444444</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 94 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 94 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (21/07/2026).</t>
+          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 97 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
         </is>
       </c>
       <c r="V9" s="8" t="inlineStr">
@@ -1162,7 +1162,7 @@
         <v>46217.80902777778</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 101 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 104 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
         </is>
       </c>
       <c r="V10" s="8" t="inlineStr">
@@ -1250,7 +1250,7 @@
         <v>46199.81041666667</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 119 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 122 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
         </is>
       </c>
       <c r="V11" s="8" t="inlineStr">
@@ -1332,7 +1332,7 @@
         <v>46181.99722222222</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 137 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 140 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
         </is>
       </c>
       <c r="V12" s="8" t="inlineStr">
@@ -1420,7 +1420,7 @@
         <v>46013.78333333333</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 305 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
+          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 308 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -1506,7 +1506,7 @@
         <v>45958.84930555556</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
@@ -1537,12 +1537,12 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 360 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 363 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 360 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
+          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 363 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
         </is>
       </c>
       <c r="V14" s="8" t="inlineStr">
@@ -1584,7 +1584,7 @@
         <v>45936.61597222222</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1615,12 +1615,12 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 382 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 385 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 382 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 385 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V15" s="8" t="inlineStr">
@@ -1662,7 +1662,7 @@
         <v>45936.87291666667</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 382 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 385 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 382 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 385 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V16" s="8" t="inlineStr">
@@ -1740,7 +1740,7 @@
         <v>45931.69513888889</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 387 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
+          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 390 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
         </is>
       </c>
       <c r="V17" s="8" t="inlineStr">
@@ -1828,7 +1828,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 472 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 475 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
         </is>
       </c>
       <c r="V18" s="8" t="inlineStr">
@@ -1916,7 +1916,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 472 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 475 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
         </is>
       </c>
       <c r="V19" s="8" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2872,20 +2872,20 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>46217.80902777778</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -2897,20 +2897,20 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>46239.78258101852</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>46239.78258101852</v>
+        <v>46217.80902777778</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -2951,16 +2951,16 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46239.78258101852</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -2976,16 +2976,16 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46239.78258101852</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3022,20 +3022,20 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>46199.81041666667</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -3047,20 +3047,20 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>46217.74835648148</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>46217.74835648148</v>
+        <v>46199.81041666667</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -3101,10 +3101,18 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>46268.96559027778</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
+        <v>46217.74835648148</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Absolución de consultas</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Pliego de absolución de consultas y observaciones</t>
+        </is>
+      </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3118,10 +3126,18 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>46268.96734953704</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
+        <v>46217.74835648148</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Bases</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Bases Integradas</t>
+        </is>
+      </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3135,18 +3151,10 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>46295.72564814815</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Presentación de Propuestas</t>
-        </is>
-      </c>
+        <v>46268.96559027778</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3160,18 +3168,10 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>46295.72565972222</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Evaluación / cuadro comparativo</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Calificación y Evaluación</t>
-        </is>
-      </c>
+        <v>46268.96734953704</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3185,16 +3185,16 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46295.72564814815</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -3206,20 +3206,20 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>46181.99722222222</v>
+        <v>46295.72565972222</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3231,20 +3231,20 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>46205.90194444444</v>
+        <v>46295.72565972222</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -3260,7 +3260,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>46205.90195601852</v>
+        <v>46181.99722222222</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -3285,16 +3285,16 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>46226.00878472222</v>
+        <v>46205.90194444444</v>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46205.90195601852</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -3335,16 +3335,16 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46226.00878472222</v>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -3356,20 +3356,20 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>46013.78333333333</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -3381,20 +3381,20 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>46021.28239583333</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Acta de no formulación de consultas y observaciones</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -3410,7 +3410,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>46021.70075231481</v>
+        <v>46013.78333333333</v>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -3435,16 +3435,16 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>46043.68869212963</v>
+        <v>46021.28239583333</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Acta de no formulación de consultas y observaciones</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -3460,16 +3460,16 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>46043.68869212963</v>
+        <v>46021.70075231481</v>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -3485,16 +3485,16 @@
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>46043.6887037037</v>
+        <v>46043.68869212963</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -3510,10 +3510,18 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>46077.64881944445</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr"/>
+        <v>46043.68869212963</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Evaluación / cuadro comparativo</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Calificación y Evaluación</t>
+        </is>
+      </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3527,7 +3535,7 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>46077.65069444444</v>
+        <v>46043.6887037037</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
@@ -3552,18 +3560,10 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>46077.6509375</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Buena pro</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
-        </is>
-      </c>
+        <v>46077.64881944445</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr"/>
       <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>46077.65246527778</v>
+        <v>46077.65069444444</v>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
@@ -3602,7 +3602,7 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>46077.67525462963</v>
+        <v>46077.6509375</v>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>46077.67789351852</v>
+        <v>46077.65246527778</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>46077.67956018518</v>
+        <v>46077.67525462963</v>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>46077.75027777778</v>
+        <v>46077.67789351852</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
@@ -3698,20 +3698,20 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B43" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>46077.67956018518</v>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -3723,20 +3723,20 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>46077.75027777778</v>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -3748,11 +3748,11 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
@@ -3773,11 +3773,11 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
@@ -3798,11 +3798,11 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Resumen ejecutivo</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -3831,12 +3831,12 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Informe que sustenta la declaratoria de Desierto</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -3852,16 +3852,16 @@
         </is>
       </c>
       <c r="B49" s="6" t="n">
-        <v>45945.71658564815</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Resumen ejecutivo</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -3877,16 +3877,16 @@
         </is>
       </c>
       <c r="B50" s="6" t="n">
-        <v>45945.71658564815</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Informe que sustenta la declaratoria de Desierto</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -3902,16 +3902,16 @@
         </is>
       </c>
       <c r="B51" s="6" t="n">
-        <v>45953.42690972222</v>
+        <v>45945.71658564815</v>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -3927,16 +3927,16 @@
         </is>
       </c>
       <c r="B52" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45945.71658564815</v>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -3952,16 +3952,16 @@
         </is>
       </c>
       <c r="B53" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45953.42690972222</v>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -3973,20 +3973,20 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B54" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -3998,20 +3998,20 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B55" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="B56" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -4052,16 +4052,16 @@
         </is>
       </c>
       <c r="B57" s="6" t="n">
-        <v>45910.79684027778</v>
+        <v>45902.81356481482</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -4077,16 +4077,16 @@
         </is>
       </c>
       <c r="B58" s="6" t="n">
-        <v>45937.76886574074</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -4102,16 +4102,16 @@
         </is>
       </c>
       <c r="B59" s="6" t="n">
-        <v>45937.76886574074</v>
+        <v>45910.79684027778</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -4127,10 +4127,18 @@
         </is>
       </c>
       <c r="B60" s="6" t="n">
-        <v>45966.75502314815</v>
-      </c>
-      <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="5" t="inlineStr"/>
+        <v>45937.76886574074</v>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Evaluación / cuadro comparativo</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Calificación y Evaluación</t>
+        </is>
+      </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4144,7 +4152,7 @@
         </is>
       </c>
       <c r="B61" s="6" t="n">
-        <v>45966.75679398148</v>
+        <v>45937.76886574074</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
@@ -4169,18 +4177,10 @@
         </is>
       </c>
       <c r="B62" s="6" t="n">
-        <v>45846.64722222222</v>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Bases Administrativas</t>
-        </is>
-      </c>
+        <v>45966.75502314815</v>
+      </c>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
       <c r="E62" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4194,16 +4194,16 @@
         </is>
       </c>
       <c r="B63" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45966.75679398148</v>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="B64" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -4244,16 +4244,16 @@
         </is>
       </c>
       <c r="B65" s="6" t="n">
-        <v>45910.79684027778</v>
+        <v>45902.81356481482</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -4269,16 +4269,16 @@
         </is>
       </c>
       <c r="B66" s="6" t="n">
-        <v>45910.79685185185</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -4294,19 +4294,69 @@
         </is>
       </c>
       <c r="B67" s="6" t="n">
+        <v>45910.79684027778</v>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Bases</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Presentación de Propuestas</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>CP-ABR-1-2025-ATU-1</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="n">
         <v>45910.79685185185</v>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Evaluación / cuadro comparativo</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Calificación y Evaluación</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>CP-ABR-1-2025-ATU-1</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="n">
+        <v>45910.79685185185</v>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Buena pro</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
-      <c r="E67" s="8" t="inlineStr">
+      <c r="E69" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4380,10 +4430,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza procesos SEACE (27/10/2026 08:30)
</commit_message>
<xml_diff>
--- a/seace/Procesos_SEACE_ATU.xlsx
+++ b/seace/Procesos_SEACE_ATU.xlsx
@@ -617,7 +617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Convocatorias desde 2025 · Revisados: 101 · Vigentes: 15 · Generado: 26/10/2026 09:35 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
+          <t>Convocatorias desde 2025 · Revisados: 101 · Vigentes: 15 · Generado: 27/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         <v>46317.78611111111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -797,12 +797,12 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Consultas y observaciones hasta el 27/10/2026 (1 días).</t>
+          <t>Consultas y observaciones hasta el 27/10/2026 (vence hoy).</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 4 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 5 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
         </is>
       </c>
       <c r="V5" s="8" t="inlineStr">
@@ -844,7 +844,7 @@
         <v>46304.93541666667</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 17 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
+          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 18 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
         </is>
       </c>
       <c r="V6" s="8" t="inlineStr">
@@ -928,7 +928,7 @@
         <v>46296.87777777778</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 25 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 26 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
         </is>
       </c>
       <c r="V7" s="8" t="inlineStr">
@@ -1006,7 +1006,7 @@
         <v>46276.85416666666</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 45 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 46 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
         </is>
       </c>
       <c r="V8" s="8" t="inlineStr">
@@ -1084,7 +1084,7 @@
         <v>46224.80069444444</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 97 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 98 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
         </is>
       </c>
       <c r="V9" s="8" t="inlineStr">
@@ -1162,7 +1162,7 @@
         <v>46217.80902777778</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 104 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 105 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
         </is>
       </c>
       <c r="V10" s="8" t="inlineStr">
@@ -1250,7 +1250,7 @@
         <v>46199.81041666667</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 122 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 123 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
         </is>
       </c>
       <c r="V11" s="8" t="inlineStr">
@@ -1332,7 +1332,7 @@
         <v>46181.99722222222</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 140 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 141 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
         </is>
       </c>
       <c r="V12" s="8" t="inlineStr">
@@ -1420,7 +1420,7 @@
         <v>46013.78333333333</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 308 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
+          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 309 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -1506,7 +1506,7 @@
         <v>45958.84930555556</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
@@ -1537,12 +1537,12 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 363 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 364 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 363 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
+          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 364 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
         </is>
       </c>
       <c r="V14" s="8" t="inlineStr">
@@ -1584,7 +1584,7 @@
         <v>45936.61597222222</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1615,12 +1615,12 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 385 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 386 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 385 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 386 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V15" s="8" t="inlineStr">
@@ -1662,7 +1662,7 @@
         <v>45936.87291666667</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 385 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 386 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 385 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 386 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V16" s="8" t="inlineStr">
@@ -1740,7 +1740,7 @@
         <v>45931.69513888889</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 390 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
+          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 391 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
         </is>
       </c>
       <c r="V17" s="8" t="inlineStr">
@@ -1828,7 +1828,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 475 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 476 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
         </is>
       </c>
       <c r="V18" s="8" t="inlineStr">
@@ -1916,7 +1916,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 475 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 476 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
         </is>
       </c>
       <c r="V19" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Actualiza procesos SEACE (28/10/2026 08:30)
</commit_message>
<xml_diff>
--- a/seace/Procesos_SEACE_ATU.xlsx
+++ b/seace/Procesos_SEACE_ATU.xlsx
@@ -219,8 +219,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Procesos" displayName="Procesos" ref="A4:V19" headerRowCount="1">
-  <autoFilter ref="A4:V19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Procesos" displayName="Procesos" ref="A4:V20" headerRowCount="1">
+  <autoFilter ref="A4:V20"/>
   <tableColumns count="22">
     <tableColumn id="1" name="N°"/>
     <tableColumn id="2" name="Nomenclatura"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Items" displayName="Items" ref="A1:H17" headerRowCount="1">
-  <autoFilter ref="A1:H17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Items" displayName="Items" ref="A1:H18" headerRowCount="1">
+  <autoFilter ref="A1:H18"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Nomenclatura"/>
     <tableColumn id="2" name="Ítem"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E69" headerRowCount="1">
-  <autoFilter ref="A1:E69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E70" headerRowCount="1">
+  <autoFilter ref="A1:E70"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Nomenclatura"/>
     <tableColumn id="2" name="Fecha publicación"/>
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -617,7 +617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Convocatorias desde 2025 · Revisados: 101 · Vigentes: 15 · Generado: 27/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
+          <t>Convocatorias desde 2025 · Revisados: 102 · Vigentes: 16 · Generado: 28/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
         </is>
       </c>
     </row>
@@ -739,12 +739,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-6-2026-ATU-1</t>
+          <t>CP-ABR-7-2026-ATU.-1</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>1260294</t>
+          <t>1261084</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -759,14 +759,14 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE GARANTIA EXTENDIDA PARA LOS SERVIDORES Y STORAGES FISICOS IMPLEMENTADOS EN LOS CENTROS DE DATOS DE LAS SEDES SURQUILLO Y CERCADO DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
+          <t>SERVICIO DE MONITOREO Y ALERTA PARA EL EQUIPO TECNOLOGICO DEL CENTRO DE DATOS DE LA UNIDAD DE TECNOLOGIA DE LA INFORMACIÓN DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>46317.78611111111</v>
+        <v>46321.88611111111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -778,10 +778,10 @@
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="6" t="n">
-        <v>46318.00069444445</v>
+        <v>46322.00069444445</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>46322.99930555555</v>
+        <v>46324.99930555555</v>
       </c>
       <c r="N5" s="4" t="n"/>
       <c r="O5" s="5" t="n"/>
@@ -793,16 +793,16 @@
         </is>
       </c>
       <c r="S5" s="6" t="n">
-        <v>46317.78611111111</v>
+        <v>46321.88611111111</v>
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Consultas y observaciones hasta el 27/10/2026 (vence hoy).</t>
+          <t>Consultas y observaciones hasta el 29/10/2026 (1 día).</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 5 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 26/10/2026 (hace 2 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (26/10/2026).</t>
         </is>
       </c>
       <c r="V5" s="8" t="inlineStr">
@@ -817,76 +817,70 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP-ABR-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>1256834</t>
+          <t>1260294</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Regímen Especial</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DIRECTA: Prestaciones pendientes para la Ejecución del saldo de la obra ¿Construcción y Adecuación de Infraestructura Interna, Externa y Zonas de Influencia Directa de la Clínica Universitaria dentro de la UNMSM</t>
+          <t>SERVICIO DE GARANTIA EXTENDIDA PARA LOS SERVIDORES Y STORAGES FISICOS IMPLEMENTADOS EN LOS CENTROS DE DATOS DE LAS SEDES SURQUILLO Y CERCADO DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>46304.93541666667</v>
+        <v>46317.78611111111</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>CONSENTIDO</t>
+        <v>6</v>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>CONSORCIO EJECUTOR SAN MARCOS</t>
-        </is>
-      </c>
-      <c r="P6" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="6" t="n">
+        <v>46318.00069444445</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>46322.99930555555</v>
+      </c>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="S6" s="6" t="n">
-        <v>46307.87658564815</v>
+        <v>46317.78611111111</v>
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
+          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 18 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 6 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
         </is>
       </c>
       <c r="V6" s="8" t="inlineStr">
@@ -901,70 +895,76 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1254828</t>
+          <t>1256834</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Regímen Especial</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Obras</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
+          <t>CONTRATACION DIRECTA: Prestaciones pendientes para la Ejecución del saldo de la obra ¿Construcción y Adecuación de Infraestructura Interna, Externa y Zonas de Influencia Directa de la Clínica Universitaria dentro de la UNMSM</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46304.93541666667</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>CONVOCADO</t>
+        <v>19</v>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="6" t="n">
-        <v>46297.00069444445</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>46309.99930555555</v>
-      </c>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="4" t="n"/>
+      <c r="K7" s="10" t="n">
+        <v>3829503.56</v>
+      </c>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>CONSORCIO EJECUTOR SAN MARCOS</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="n">
+        <v>3829503.56</v>
+      </c>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="S7" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46307.87658564815</v>
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
+          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 26 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
+          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 19 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
         </is>
       </c>
       <c r="V7" s="8" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1249681</t>
+          <t>1254828</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -999,14 +999,14 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
+          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -1018,10 +1018,10 @@
       </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="6" t="n">
-        <v>46277.00069444445</v>
+        <v>46297.00069444445</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>46287.99930555555</v>
+        <v>46309.99930555555</v>
       </c>
       <c r="N8" s="4" t="n"/>
       <c r="O8" s="5" t="n"/>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="S8" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 46 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 27 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
         </is>
       </c>
       <c r="V8" s="8" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>1235886</t>
+          <t>1249681</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1077,14 +1077,14 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
+          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46224.80069444444</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
@@ -1096,10 +1096,10 @@
       </c>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="6" t="n">
-        <v>46225.00069444445</v>
+        <v>46277.00069444445</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>46239.99930555555</v>
+        <v>46287.99930555555</v>
       </c>
       <c r="N9" s="4" t="n"/>
       <c r="O9" s="5" t="n"/>
@@ -1107,11 +1107,11 @@
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="S9" s="6" t="n">
-        <v>46318.75248842593</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 98 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 47 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
         </is>
       </c>
       <c r="V9" s="8" t="inlineStr">
@@ -1135,17 +1135,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1233921</t>
+          <t>1235886</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1155,60 +1155,50 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
+          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>46217.80902777778</v>
+        <v>46224.80069444444</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
+        <v>99</v>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="10" t="n">
-        <v>481750</v>
-      </c>
+      <c r="K10" s="4" t="n"/>
       <c r="L10" s="6" t="n">
-        <v>46218.00069444445</v>
+        <v>46225.00069444445</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>46220.99930555555</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>LOGISTAS SERVICIOS S.A.C.</t>
-        </is>
-      </c>
-      <c r="P10" s="10" t="n">
-        <v>315952</v>
-      </c>
+        <v>46239.99930555555</v>
+      </c>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="S10" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>En trámite: pendiente de registro de efecto.</t>
+          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 105 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
+          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 99 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
         </is>
       </c>
       <c r="V10" s="8" t="inlineStr">
@@ -1223,17 +1213,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1229354</t>
+          <t>1233921</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1243,37 +1233,43 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
+          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46199.81041666667</v>
+        <v>46217.80902777778</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>123</v>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>APELADO</t>
+        <v>106</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>3565508.55</v>
+        <v>481750</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>46200.00069444445</v>
+        <v>46218.00069444445</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>46211.99930555555</v>
+        <v>46220.99930555555</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O11" s="5" t="n"/>
-      <c r="P11" s="4" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>LOGISTAS SERVICIOS S.A.C.</t>
+        </is>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>315952</v>
+      </c>
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="5" t="inlineStr">
         <is>
@@ -1281,16 +1277,16 @@
         </is>
       </c>
       <c r="S11" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>En apelación: hacer seguimiento a la resolución del recurso.</t>
+          <t>En trámite: pendiente de registro de efecto.</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 123 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 106 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
         </is>
       </c>
       <c r="V11" s="8" t="inlineStr">
@@ -1305,63 +1301,57 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>1223446</t>
+          <t>1229354</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 - CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE, LA VICTORIA, SAN BORJA, SANTIAGO DE SURCO, ATE</t>
+          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>46181.99722222222</v>
+        <v>46199.81041666667</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>141</v>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        <v>124</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>APELADO</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K12" s="10" t="n">
-        <v>4933726.01</v>
+        <v>3565508.55</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>46182.00069444445</v>
+        <v>46200.00069444445</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>46184.99930555555</v>
+        <v>46211.99930555555</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>64</v>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>CONSORCIO PROGRESO</t>
-        </is>
-      </c>
-      <c r="P12" s="10" t="n">
-        <v>4687039.71</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="5" t="inlineStr">
         <is>
@@ -1369,16 +1359,16 @@
         </is>
       </c>
       <c r="S12" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46295.72565972222</v>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
+          <t>En apelación: hacer seguimiento a la resolución del recurso.</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 141 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
+          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 124 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
         </is>
       </c>
       <c r="V12" s="8" t="inlineStr">
@@ -1393,12 +1383,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>1180205</t>
+          <t>1223446</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1408,45 +1398,47 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Bienes</t>
+          <t>Obras</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALDOSAS PODOTACTILES ADOSABLES PARA LAS ESTACIONES DEL COSAC I</t>
+          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 - CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE, LA VICTORIA, SAN BORJA, SANTIAGO DE SURCO, ATE</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>46013.78333333333</v>
+        <v>46181.99722222222</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>309</v>
+        <v>142</v>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>CONVOCADO_POR_REINICIO</t>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="K13" s="10" t="n">
+        <v>4933726.01</v>
+      </c>
       <c r="L13" s="6" t="n">
-        <v>46014.00069444445</v>
+        <v>46182.00069444445</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>46020.99930555555</v>
+        <v>46184.99930555555</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>SOLUCIONES ESPECIALES S.A.C.</t>
+          <t>CONSORCIO PROGRESO</t>
         </is>
       </c>
       <c r="P13" s="10" t="n">
-        <v>468000</v>
+        <v>4687039.71</v>
       </c>
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="5" t="inlineStr">
@@ -1455,7 +1447,7 @@
         </is>
       </c>
       <c r="S13" s="6" t="n">
-        <v>46077.75027777778</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
@@ -1464,7 +1456,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 309 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 142 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -1479,70 +1471,78 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>1164719</t>
+          <t>1180205</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Licitación Pública Abreviada</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Bienes</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
+          <t>ADQUISICION DE BALDOSAS PODOTACTILES ADOSABLES PARA LAS ESTACIONES DEL COSAC I</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>46013.78333333333</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>364</v>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>CONVOCADO</t>
+        <v>310</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>CONVOCADO_POR_REINICIO</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="6" t="n">
-        <v>45959.00069444445</v>
+        <v>46014.00069444445</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>45972.99930555555</v>
-      </c>
-      <c r="N14" s="4" t="n"/>
-      <c r="O14" s="5" t="n"/>
-      <c r="P14" s="4" t="n"/>
+        <v>46020.99930555555</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>SOLUCIONES ESPECIALES S.A.C.</t>
+        </is>
+      </c>
+      <c r="P14" s="10" t="n">
+        <v>468000</v>
+      </c>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="S14" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>46077.75027777778</v>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 364 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 364 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
+          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 310 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
         </is>
       </c>
       <c r="V14" s="8" t="inlineStr">
@@ -1557,17 +1557,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>1157662</t>
+          <t>1164719</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1577,14 +1577,14 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
+          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>386</v>
+        <v>365</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1596,10 +1596,10 @@
       </c>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="6" t="n">
-        <v>45937.00069444445</v>
+        <v>45959.00069444445</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>45940.99930555555</v>
+        <v>45972.99930555555</v>
       </c>
       <c r="N15" s="4" t="n"/>
       <c r="O15" s="5" t="n"/>
@@ -1611,16 +1611,16 @@
         </is>
       </c>
       <c r="S15" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 386 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 365 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 386 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 365 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
         </is>
       </c>
       <c r="V15" s="8" t="inlineStr">
@@ -1635,34 +1635,34 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>1157850</t>
+          <t>1157662</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DIST</t>
+          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="S16" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 386 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 387 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 386 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 387 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V16" s="8" t="inlineStr">
@@ -1713,80 +1713,70 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>1156331</t>
+          <t>1157850</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada</t>
+          <t>Licitación Pública Abreviada</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Bienes</t>
+          <t>Obras</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición e instalación de grupo electrógeno insonoro de 250 KVA para la sede Lima de la Autoridad de Transporte Urbano para Lima y Callao</t>
+          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DIST</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>391</v>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>CONSENTIDO</t>
+        <v>387</v>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="10" t="n">
-        <v>395000</v>
-      </c>
+      <c r="K17" s="4" t="n"/>
       <c r="L17" s="6" t="n">
-        <v>45932.00069444445</v>
+        <v>45937.00069444445</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>45936.99930555555</v>
-      </c>
-      <c r="N17" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O17" s="5" t="inlineStr">
-        <is>
-          <t>SERVFAC PERU E.I.R.L.</t>
-        </is>
-      </c>
-      <c r="P17" s="10" t="n">
-        <v>378900</v>
-      </c>
+        <v>45940.99930555555</v>
+      </c>
+      <c r="N17" s="4" t="n"/>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="4" t="n"/>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="S17" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
+          <t>Convocado sin documentos nuevos hace 387 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 391 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 387 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V17" s="8" t="inlineStr">
@@ -1801,62 +1791,62 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>1157235</t>
+          <t>1156331</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado</t>
+          <t>Adjudicación Simplificada</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Bienes</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
+          <t>Adquisición e instalación de grupo electrógeno insonoro de 250 KVA para la sede Lima de la Autoridad de Transporte Urbano para Lima y Callao</t>
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>476</v>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        <v>392</v>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="10" t="n">
-        <v>278000</v>
+        <v>395000</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>45847.00069444445</v>
+        <v>45932.00069444445</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>45849.99930555555</v>
+        <v>45936.99930555555</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>GATT PERU S.R.L.; HERMES GROUP SAC</t>
+          <t>SERVFAC PERU E.I.R.L.</t>
         </is>
       </c>
       <c r="P18" s="10" t="n">
-        <v>488990</v>
+        <v>378900</v>
       </c>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="5" t="inlineStr">
@@ -1865,16 +1855,16 @@
         </is>
       </c>
       <c r="S18" s="6" t="n">
-        <v>45966.75679398148</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
+          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 476 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 392 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
         </is>
       </c>
       <c r="V18" s="8" t="inlineStr">
@@ -1894,7 +1884,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>1131459</t>
+          <t>1157235</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1916,7 +1906,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
@@ -1936,15 +1926,15 @@
         <v>45849.99930555555</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>GATT PERU S.R.L.</t>
+          <t>GATT PERU S.R.L.; HERMES GROUP SAC</t>
         </is>
       </c>
       <c r="P19" s="10" t="n">
-        <v>248990</v>
+        <v>488990</v>
       </c>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="5" t="inlineStr">
@@ -1953,19 +1943,107 @@
         </is>
       </c>
       <c r="S19" s="6" t="n">
+        <v>45966.75679398148</v>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
+        </is>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 477 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+        </is>
+      </c>
+      <c r="V19" s="8" t="inlineStr">
+        <is>
+          <t>Ver proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>CP-ABR-1-2025-ATU-1</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>1131459</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Concurso Público Abreviado</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>45846.64722222222</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>477</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>278000</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>45847.00069444445</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>45849.99930555555</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>GATT PERU S.R.L.</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="n">
+        <v>248990</v>
+      </c>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
+        </is>
+      </c>
+      <c r="S20" s="6" t="n">
         <v>45910.79685185185</v>
       </c>
-      <c r="T19" s="5" t="inlineStr">
+      <c r="T20" s="5" t="inlineStr">
         <is>
           <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
         </is>
       </c>
-      <c r="U19" s="5" t="inlineStr">
-        <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 476 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
-        </is>
-      </c>
-      <c r="V19" s="8" t="inlineStr">
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 477 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
+        </is>
+      </c>
+      <c r="V20" s="8" t="inlineStr">
         <is>
           <t>Ver proceso</t>
         </is>
@@ -1988,10 +2066,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2002,7 +2081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2060,7 +2139,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-6-2026-ATU-1</t>
+          <t>CP-ABR-7-2026-ATU.-1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -2070,7 +2149,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE GARANTIA EXTENDIDA PARA LOS SERVIDORES Y STORAGES FISICOS IMPLEMENTADOS EN LOS CENTROS DE DATOS DE LAS SEDES SURQUILLO Y CERCADO DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
+          <t>SERVICIO DE MONITOREO Y ALERTA PARA EL EQUIPO TECNOLOGICO DEL CENTRO DE DATOS DE LA UNIDAD DE TECNOLOGIA DE LA INFORMACIÓN DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -2089,14 +2168,14 @@
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE GARANTIA EXTENDIDA</t>
+          <t>SERVICIO DE SOPORTE TECNICO PARA EQUIPOS TECNOLOGICOS DE LA INFORMACION</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP-ABR-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -2106,12 +2185,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>PRESTACIONES PENDIENTES PARA LA EJECUCION DEL SALDO DE OBRA DEL PROYECTO CONSTRUCCIÓN Y ADECUACIÓN DE INFRAESTRUCTURA INTERNA, EXTERNA Y ZONAS DE INFLUENCIA DIRECTA DE LA CLÍNICA UNIVERSITARIA DENTRO DE LA UNMSM¿PRESTACIONES PENDIENTES PARA LA EJEC</t>
+          <t>SERVICIO DE GARANTIA EXTENDIDA PARA LOS SERVIDORES Y STORAGES FISICOS IMPLEMENTADOS EN LOS CENTROS DE DATOS DE LAS SEDES SURQUILLO Y CERCADO DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO - ATU</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>CONSENTIDO</t>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
@@ -2122,19 +2201,17 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G3" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
+      <c r="G3" s="4" t="n"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE INFRAESTRUCTURA DE SALUD</t>
+          <t>SERVICIO DE GARANTIA EXTENDIDA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -2144,12 +2221,12 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
+          <t>PRESTACIONES PENDIENTES PARA LA EJECUCION DEL SALDO DE OBRA DEL PROYECTO CONSTRUCCIÓN Y ADECUACIÓN DE INFRAESTRUCTURA INTERNA, EXTERNA Y ZONAS DE INFLUENCIA DIRECTA DE LA CLÍNICA UNIVERSITARIA DENTRO DE LA UNMSM¿PRESTACIONES PENDIENTES PARA LA EJEC</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO</t>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
@@ -2160,17 +2237,19 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G4" s="4" t="n"/>
+      <c r="G4" s="10" t="n">
+        <v>3829503.56</v>
+      </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>RENOVACION DEL SOPORTE Y MANTENIMIENTO DE LICENCIAS DE SOFTWARE PARA EL ERP SAP</t>
+          <t>CONSTRUCCION DE INFRAESTRUCTURA DE SALUD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -2180,7 +2259,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
+          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2193,16 +2272,20 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Servicio</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>RENOVACION DEL SOPORTE Y MANTENIMIENTO DE LICENCIAS DE SOFTWARE PARA EL ERP SAP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2212,7 +2295,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
+          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2225,20 +2308,16 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE CABLEADO ESTRUCTURADO Y CONEXION DE FIBRA OPTICA</t>
-        </is>
-      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2248,12 +2327,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
+          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
@@ -2264,19 +2343,17 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G7" s="10" t="n">
-        <v>481750</v>
-      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE GRUA</t>
+          <t>SERVICIO DE CABLEADO ESTRUCTURADO Y CONEXION DE FIBRA OPTICA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2286,12 +2363,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
+          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>APELADO</t>
+          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
@@ -2303,33 +2380,33 @@
         </is>
       </c>
       <c r="G8" s="10" t="n">
-        <v>3565508.55</v>
+        <v>481750</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE VEHICULOS</t>
+          <t>SERVICIO DE ALQUILER DE GRUA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 -CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE</t>
+          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
+          <t>APELADO</t>
         </is>
       </c>
       <c r="E9" s="10" t="n">
@@ -2341,47 +2418,49 @@
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>4933726.01</v>
+        <v>3565508.55</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE CARRETERA</t>
+          <t>SERVICIO DE ALQUILER DE VEHICULOS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>BALDOSA PODOTACTIL DE GUIA</t>
+          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 -CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO_POR_REINICIO</t>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n"/>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>4933726.01</v>
+      </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>PISO DE JEBE DE 4 mm X 0.40 m X 0.60 m</t>
+          <t>CONSTRUCCION DE CARRETERA</t>
         </is>
       </c>
     </row>
@@ -2393,12 +2472,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>BALDOSA PODOTACTIL DE ALERTA</t>
+          <t>BALDOSA PODOTACTIL DE GUIA</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -2407,7 +2486,7 @@
         </is>
       </c>
       <c r="E11" s="10" t="n">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
@@ -2424,7 +2503,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2434,33 +2513,33 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
+          <t>BALDOSA PODOTACTIL DE ALERTA</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO</t>
+          <t>CONVOCADO_POR_REINICIO</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD Y VIGILANCIA</t>
+          <t>PISO DE JEBE DE 4 mm X 0.40 m X 0.60 m</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -2470,7 +2549,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
+          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2489,14 +2568,14 @@
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO DE PUERTAS LEVADIZAS</t>
+          <t>SERVICIO DE SEGURIDAD Y VIGILANCIA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -2506,7 +2585,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RE</t>
+          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2525,14 +2604,14 @@
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE ESTACION PARA EMBARQUE DE PASAJEROS DE TRANSPORTE URBANO</t>
+          <t>SERVICIO DE MANTENIMIENTO DE PUERTAS LEVADIZAS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -2542,12 +2621,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
+          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RE</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>CONSENTIDO</t>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="E15" s="10" t="n">
@@ -2555,22 +2634,20 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>395000</v>
-      </c>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
+          <t>CONSTRUCCION DE ESTACION PARA EMBARQUE DE PASAJEROS DE TRANSPORTE URBANO</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2580,12 +2657,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
+          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="E16" s="10" t="n">
@@ -2593,15 +2670,15 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>278000</v>
+        <v>395000</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
+          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
         </is>
       </c>
     </row>
@@ -2638,6 +2715,44 @@
         <v>278000</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CP-ABR-1-2025-ATU-1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>278000</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
         </is>
@@ -2657,7 +2772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2697,11 +2812,11 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-6-2026-ATU-1</t>
+          <t>CP-ABR-7-2026-ATU.-1</t>
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>46317.78611111111</v>
+        <v>46321.88611111111</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -2722,11 +2837,11 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP-ABR-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>46304.93541666667</v>
+        <v>46317.78611111111</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -2751,7 +2866,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>46307.87658564815</v>
+        <v>46304.93541666667</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -2760,7 +2875,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -2780,12 +2895,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -2797,20 +2912,20 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46307.87658564815</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -2822,11 +2937,11 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -2847,11 +2962,11 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>46224.80069444444</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -2876,16 +2991,16 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>46318.75248842593</v>
+        <v>46224.80069444444</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -2905,12 +3020,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -2922,11 +3037,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>46217.80902777778</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -2935,7 +3050,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -2951,16 +3066,16 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>46239.78258101852</v>
+        <v>46217.80902777778</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -2980,12 +3095,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -3001,7 +3116,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46239.78258101852</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
@@ -3010,7 +3125,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3030,12 +3145,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -3055,12 +3170,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -3072,20 +3187,20 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>46199.81041666667</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -3101,16 +3216,16 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>46217.74835648148</v>
+        <v>46199.81041666667</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -3130,12 +3245,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -3151,10 +3266,18 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>46268.96559027778</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
+        <v>46217.74835648148</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Bases</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Bases Integradas</t>
+        </is>
+      </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3168,7 +3291,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>46268.96734953704</v>
+        <v>46268.96559027778</v>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="5" t="inlineStr"/>
@@ -3185,18 +3308,10 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>46295.72564814815</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Presentación de Propuestas</t>
-        </is>
-      </c>
+        <v>46268.96734953704</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3210,16 +3325,16 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46295.72564814815</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3239,12 +3354,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -3256,20 +3371,20 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>46181.99722222222</v>
+        <v>46295.72565972222</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -3285,16 +3400,16 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>46205.90194444444</v>
+        <v>46181.99722222222</v>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -3310,16 +3425,16 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>46205.90195601852</v>
+        <v>46205.90194444444</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -3335,7 +3450,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>46226.00878472222</v>
+        <v>46205.90195601852</v>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
@@ -3344,7 +3459,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -3360,16 +3475,16 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46226.00878472222</v>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -3389,12 +3504,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -3406,20 +3521,20 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>46013.78333333333</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -3435,16 +3550,16 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>46021.28239583333</v>
+        <v>46013.78333333333</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Acta de no formulación de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -3460,16 +3575,16 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>46021.70075231481</v>
+        <v>46021.28239583333</v>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Acta de no formulación de consultas y observaciones</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -3485,7 +3600,7 @@
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>46043.68869212963</v>
+        <v>46021.70075231481</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
@@ -3494,7 +3609,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -3514,12 +3629,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -3535,16 +3650,16 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>46043.6887037037</v>
+        <v>46043.68869212963</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -3560,10 +3675,18 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>46077.64881944445</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr"/>
+        <v>46043.6887037037</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Buena pro</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
+        </is>
+      </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3577,18 +3700,10 @@
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>46077.65069444444</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Buena pro</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
-        </is>
-      </c>
+        <v>46077.64881944445</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr"/>
       <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3602,7 +3717,7 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>46077.6509375</v>
+        <v>46077.65069444444</v>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
@@ -3627,7 +3742,7 @@
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>46077.65246527778</v>
+        <v>46077.6509375</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
@@ -3652,7 +3767,7 @@
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>46077.67525462963</v>
+        <v>46077.65246527778</v>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
@@ -3677,7 +3792,7 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>46077.67789351852</v>
+        <v>46077.67525462963</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
@@ -3702,7 +3817,7 @@
         </is>
       </c>
       <c r="B43" s="6" t="n">
-        <v>46077.67956018518</v>
+        <v>46077.67789351852</v>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
@@ -3727,7 +3842,7 @@
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>46077.75027777778</v>
+        <v>46077.67956018518</v>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
@@ -3748,20 +3863,20 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>46077.75027777778</v>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -3773,11 +3888,11 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
@@ -3798,11 +3913,11 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
@@ -3823,11 +3938,11 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="B48" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
@@ -3861,7 +3976,7 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Resumen ejecutivo</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -3881,12 +3996,12 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Informe que sustenta la declaratoria de Desierto</t>
+          <t>Resumen ejecutivo</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -3902,16 +4017,16 @@
         </is>
       </c>
       <c r="B51" s="6" t="n">
-        <v>45945.71658564815</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Informe que sustenta la declaratoria de Desierto</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -3931,12 +4046,12 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -3952,7 +4067,7 @@
         </is>
       </c>
       <c r="B53" s="6" t="n">
-        <v>45953.42690972222</v>
+        <v>45945.71658564815</v>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
@@ -3961,7 +4076,7 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -3977,16 +4092,16 @@
         </is>
       </c>
       <c r="B54" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45953.42690972222</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -4006,12 +4121,12 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -4023,20 +4138,20 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B56" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -4052,16 +4167,16 @@
         </is>
       </c>
       <c r="B57" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -4077,16 +4192,16 @@
         </is>
       </c>
       <c r="B58" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45902.81356481482</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -4102,7 +4217,7 @@
         </is>
       </c>
       <c r="B59" s="6" t="n">
-        <v>45910.79684027778</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
@@ -4111,7 +4226,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -4127,16 +4242,16 @@
         </is>
       </c>
       <c r="B60" s="6" t="n">
-        <v>45937.76886574074</v>
+        <v>45910.79684027778</v>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -4156,12 +4271,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -4177,10 +4292,18 @@
         </is>
       </c>
       <c r="B62" s="6" t="n">
-        <v>45966.75502314815</v>
-      </c>
-      <c r="C62" s="4" t="inlineStr"/>
-      <c r="D62" s="5" t="inlineStr"/>
+        <v>45937.76886574074</v>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Buena pro</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
+        </is>
+      </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4194,18 +4317,10 @@
         </is>
       </c>
       <c r="B63" s="6" t="n">
-        <v>45966.75679398148</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Buena pro</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
-        </is>
-      </c>
+        <v>45966.75502314815</v>
+      </c>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr"/>
       <c r="E63" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4219,16 +4334,16 @@
         </is>
       </c>
       <c r="B64" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45966.75679398148</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -4244,16 +4359,16 @@
         </is>
       </c>
       <c r="B65" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -4269,16 +4384,16 @@
         </is>
       </c>
       <c r="B66" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45902.81356481482</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -4294,7 +4409,7 @@
         </is>
       </c>
       <c r="B67" s="6" t="n">
-        <v>45910.79684027778</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
@@ -4303,7 +4418,7 @@
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -4319,16 +4434,16 @@
         </is>
       </c>
       <c r="B68" s="6" t="n">
-        <v>45910.79685185185</v>
+        <v>45910.79684027778</v>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -4348,15 +4463,40 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
+          <t>Evaluación / cuadro comparativo</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Calificación y Evaluación</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>CP-ABR-1-2025-ATU-1</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="n">
+        <v>45910.79685185185</v>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
           <t>Buena pro</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr">
+      <c r="E70" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4432,10 +4572,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4472,7 +4613,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Actualiza procesos SEACE (29/10/2026 08:30)
</commit_message>
<xml_diff>
--- a/seace/Procesos_SEACE_ATU.xlsx
+++ b/seace/Procesos_SEACE_ATU.xlsx
@@ -68,17 +68,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,10 +130,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -219,8 +219,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Procesos" displayName="Procesos" ref="A4:V20" headerRowCount="1">
-  <autoFilter ref="A4:V20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Procesos" displayName="Procesos" ref="A4:V19" headerRowCount="1">
+  <autoFilter ref="A4:V19"/>
   <tableColumns count="22">
     <tableColumn id="1" name="N°"/>
     <tableColumn id="2" name="Nomenclatura"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Items" displayName="Items" ref="A1:H18" headerRowCount="1">
-  <autoFilter ref="A1:H18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Items" displayName="Items" ref="A1:H17" headerRowCount="1">
+  <autoFilter ref="A1:H17"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Nomenclatura"/>
     <tableColumn id="2" name="Ítem"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E70" headerRowCount="1">
-  <autoFilter ref="A1:E70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Documentos" displayName="Documentos" ref="A1:E67" headerRowCount="1">
+  <autoFilter ref="A1:E67"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Nomenclatura"/>
     <tableColumn id="2" name="Fecha publicación"/>
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -617,7 +617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Convocatorias desde 2025 · Revisados: 102 · Vigentes: 16 · Generado: 28/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
+          <t>Convocatorias desde 2025 · Revisados: 102 · Vigentes: 15 · Generado: 29/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         <v>46321.88611111111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -797,12 +797,12 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Consultas y observaciones hasta el 29/10/2026 (1 día).</t>
+          <t>Consultas y observaciones hasta el 29/10/2026 (vence hoy).</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 26/10/2026 (hace 2 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (26/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 26/10/2026 (hace 3 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (26/10/2026).</t>
         </is>
       </c>
       <c r="V5" s="8" t="inlineStr">
@@ -844,7 +844,7 @@
         <v>46317.78611111111</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 6 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 7 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
         </is>
       </c>
       <c r="V6" s="8" t="inlineStr">
@@ -895,76 +895,70 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1256834</t>
+          <t>1254828</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Regímen Especial</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DIRECTA: Prestaciones pendientes para la Ejecución del saldo de la obra ¿Construcción y Adecuación de Infraestructura Interna, Externa y Zonas de Influencia Directa de la Clínica Universitaria dentro de la UNMSM</t>
+          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46304.93541666667</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>CONSENTIDO</t>
+        <v>28</v>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>CONSORCIO EJECUTOR SAN MARCOS</t>
-        </is>
-      </c>
-      <c r="P7" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="6" t="n">
+        <v>46297.00069444445</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>46309.99930555555</v>
+      </c>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="S7" s="6" t="n">
-        <v>46307.87658564815</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
+          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Regímen Especial de obras convocado el 09/10/2026 (hace 19 días). Valor estimado/referencial: S/ 3,829,503.56. Estado: CONSENTIDO. Postores: 2. Buena pro a CONSORCIO EJECUTOR SAN MARCOS por S/ 3,829,503.56. Último documento: Documentos de Otorgamiento de Buena Pro (12/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 28 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
         </is>
       </c>
       <c r="V7" s="8" t="inlineStr">
@@ -979,12 +973,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1254828</t>
+          <t>1249681</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -999,14 +993,14 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
+          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -1018,10 +1012,10 @@
       </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="6" t="n">
-        <v>46297.00069444445</v>
+        <v>46277.00069444445</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>46309.99930555555</v>
+        <v>46287.99930555555</v>
       </c>
       <c r="N8" s="4" t="n"/>
       <c r="O8" s="5" t="n"/>
@@ -1033,7 +1027,7 @@
         </is>
       </c>
       <c r="S8" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
@@ -1042,7 +1036,7 @@
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 27 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 48 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
         </is>
       </c>
       <c r="V8" s="8" t="inlineStr">
@@ -1057,12 +1051,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>1249681</t>
+          <t>1235886</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1077,14 +1071,14 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
+          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46224.80069444444</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
@@ -1096,10 +1090,10 @@
       </c>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="6" t="n">
-        <v>46277.00069444445</v>
+        <v>46225.00069444445</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>46287.99930555555</v>
+        <v>46239.99930555555</v>
       </c>
       <c r="N9" s="4" t="n"/>
       <c r="O9" s="5" t="n"/>
@@ -1107,11 +1101,11 @@
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="S9" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
@@ -1120,7 +1114,7 @@
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 47 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 100 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
         </is>
       </c>
       <c r="V9" s="8" t="inlineStr">
@@ -1135,17 +1129,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1235886</t>
+          <t>1233921</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1155,50 +1149,60 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
+          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>46224.80069444444</v>
+        <v>46217.80902777778</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>CONVOCADO</t>
+        <v>107</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="4" t="n"/>
+      <c r="K10" s="9" t="n">
+        <v>481750</v>
+      </c>
       <c r="L10" s="6" t="n">
-        <v>46225.00069444445</v>
+        <v>46218.00069444445</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>46239.99930555555</v>
-      </c>
-      <c r="N10" s="4" t="n"/>
-      <c r="O10" s="5" t="n"/>
-      <c r="P10" s="4" t="n"/>
+        <v>46220.99930555555</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>LOGISTAS SERVICIOS S.A.C.</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>315952</v>
+      </c>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="S10" s="6" t="n">
-        <v>46318.75248842593</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
+          <t>En trámite: pendiente de registro de efecto.</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 99 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 107 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
         </is>
       </c>
       <c r="V10" s="8" t="inlineStr">
@@ -1213,17 +1217,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1233921</t>
+          <t>1229354</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1233,43 +1237,37 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
+          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46217.80902777778</v>
+        <v>46199.81041666667</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>106</v>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
+        <v>125</v>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>APELADO</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>481750</v>
+      <c r="K11" s="9" t="n">
+        <v>3565508.55</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>46218.00069444445</v>
+        <v>46200.00069444445</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>46220.99930555555</v>
+        <v>46211.99930555555</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>LOGISTAS SERVICIOS S.A.C.</t>
-        </is>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>315952</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="5" t="inlineStr">
         <is>
@@ -1277,16 +1275,16 @@
         </is>
       </c>
       <c r="S11" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46295.72565972222</v>
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>En trámite: pendiente de registro de efecto.</t>
+          <t>En apelación: hacer seguimiento a la resolución del recurso.</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 106 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
+          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 125 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
         </is>
       </c>
       <c r="V11" s="8" t="inlineStr">
@@ -1301,57 +1299,63 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>1229354</t>
+          <t>1223446</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Licitación Pública Abreviada</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Obras</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
+          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 - CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE, LA VICTORIA, SAN BORJA, SANTIAGO DE SURCO, ATE</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>46199.81041666667</v>
+        <v>46181.99722222222</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>APELADO</t>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="10" t="n">
-        <v>3565508.55</v>
+      <c r="K12" s="9" t="n">
+        <v>4933726.01</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>46200.00069444445</v>
+        <v>46182.00069444445</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>46211.99930555555</v>
+        <v>46184.99930555555</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O12" s="5" t="n"/>
-      <c r="P12" s="4" t="n"/>
+        <v>64</v>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>CONSORCIO PROGRESO</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>4687039.71</v>
+      </c>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="5" t="inlineStr">
         <is>
@@ -1359,16 +1363,16 @@
         </is>
       </c>
       <c r="S12" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>En apelación: hacer seguimiento a la resolución del recurso.</t>
+          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 124 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 143 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
         </is>
       </c>
       <c r="V12" s="8" t="inlineStr">
@@ -1383,12 +1387,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>1223446</t>
+          <t>1180205</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1398,47 +1402,45 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Bienes</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 - CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE, LA VICTORIA, SAN BORJA, SANTIAGO DE SURCO, ATE</t>
+          <t>ADQUISICION DE BALDOSAS PODOTACTILES ADOSABLES PARA LAS ESTACIONES DEL COSAC I</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>46181.99722222222</v>
+        <v>46013.78333333333</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>142</v>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        <v>311</v>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>CONVOCADO_POR_REINICIO</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="10" t="n">
-        <v>4933726.01</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K13" s="4" t="n"/>
       <c r="L13" s="6" t="n">
-        <v>46182.00069444445</v>
+        <v>46014.00069444445</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>46184.99930555555</v>
+        <v>46020.99930555555</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>CONSORCIO PROGRESO</t>
-        </is>
-      </c>
-      <c r="P13" s="10" t="n">
-        <v>4687039.71</v>
+          <t>SOLUCIONES ESPECIALES S.A.C.</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>468000</v>
       </c>
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="5" t="inlineStr">
@@ -1447,7 +1449,7 @@
         </is>
       </c>
       <c r="S13" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46077.75027777778</v>
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
@@ -1456,7 +1458,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 142 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
+          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 311 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -1471,78 +1473,70 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>1180205</t>
+          <t>1164719</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada</t>
+          <t>Concurso Público de Servicios</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Bienes</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALDOSAS PODOTACTILES ADOSABLES PARA LAS ESTACIONES DEL COSAC I</t>
+          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>46013.78333333333</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>CONVOCADO_POR_REINICIO</t>
+        <v>366</v>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>CONVOCADO</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="6" t="n">
-        <v>46014.00069444445</v>
+        <v>45959.00069444445</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>46020.99930555555</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>SOLUCIONES ESPECIALES S.A.C.</t>
-        </is>
-      </c>
-      <c r="P14" s="10" t="n">
-        <v>468000</v>
-      </c>
+        <v>45972.99930555555</v>
+      </c>
+      <c r="N14" s="4" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="S14" s="6" t="n">
-        <v>46077.75027777778</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
+          <t>Convocado sin documentos nuevos hace 366 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 310 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
+          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 366 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
         </is>
       </c>
       <c r="V14" s="8" t="inlineStr">
@@ -1557,17 +1551,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>1164719</t>
+          <t>1157662</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1577,14 +1571,14 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
+          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>365</v>
+        <v>388</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1596,10 +1590,10 @@
       </c>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="6" t="n">
-        <v>45959.00069444445</v>
+        <v>45937.00069444445</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>45972.99930555555</v>
+        <v>45940.99930555555</v>
       </c>
       <c r="N15" s="4" t="n"/>
       <c r="O15" s="5" t="n"/>
@@ -1611,16 +1605,16 @@
         </is>
       </c>
       <c r="S15" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 365 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 388 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 365 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 388 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V15" s="8" t="inlineStr">
@@ -1635,34 +1629,34 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>1157662</t>
+          <t>1157850</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado</t>
+          <t>Licitación Pública Abreviada</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Obras</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
+          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DIST</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -1689,16 +1683,16 @@
         </is>
       </c>
       <c r="S16" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 387 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 388 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 387 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 388 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V16" s="8" t="inlineStr">
@@ -1713,70 +1707,80 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>1157850</t>
+          <t>1156331</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada</t>
+          <t>Adjudicación Simplificada</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Bienes</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DIST</t>
+          <t>Adquisición e instalación de grupo electrógeno insonoro de 250 KVA para la sede Lima de la Autoridad de Transporte Urbano para Lima y Callao</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>387</v>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>CONVOCADO</t>
+        <v>393</v>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="4" t="n"/>
+      <c r="K17" s="9" t="n">
+        <v>395000</v>
+      </c>
       <c r="L17" s="6" t="n">
-        <v>45937.00069444445</v>
+        <v>45932.00069444445</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>45940.99930555555</v>
-      </c>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="5" t="n"/>
-      <c r="P17" s="4" t="n"/>
+        <v>45936.99930555555</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>SERVFAC PERU E.I.R.L.</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="n">
+        <v>378900</v>
+      </c>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="S17" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 387 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
         </is>
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 387 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 393 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
         </is>
       </c>
       <c r="V17" s="8" t="inlineStr">
@@ -1791,62 +1795,62 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-1-2025-ATU-1</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>1156331</t>
+          <t>1157235</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada</t>
+          <t>Concurso Público Abreviado</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Bienes</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición e instalación de grupo electrógeno insonoro de 250 KVA para la sede Lima de la Autoridad de Transporte Urbano para Lima y Callao</t>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>CONSENTIDO</t>
+        <v>478</v>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="10" t="n">
-        <v>395000</v>
+      <c r="K18" s="9" t="n">
+        <v>278000</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>45932.00069444445</v>
+        <v>45847.00069444445</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>45936.99930555555</v>
+        <v>45849.99930555555</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>SERVFAC PERU E.I.R.L.</t>
-        </is>
-      </c>
-      <c r="P18" s="10" t="n">
-        <v>378900</v>
+          <t>GATT PERU S.R.L.; HERMES GROUP SAC</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="n">
+        <v>488990</v>
       </c>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="5" t="inlineStr">
@@ -1855,16 +1859,16 @@
         </is>
       </c>
       <c r="S18" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45966.75679398148</v>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Buena pro consentida: pendiente suscripción de contrato.</t>
+          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 392 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 478 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
         </is>
       </c>
       <c r="V18" s="8" t="inlineStr">
@@ -1884,7 +1888,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>1157235</t>
+          <t>1131459</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1906,9 +1910,9 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>477</v>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
+        <v>478</v>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
@@ -1916,7 +1920,7 @@
       <c r="J19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K19" s="10" t="n">
+      <c r="K19" s="9" t="n">
         <v>278000</v>
       </c>
       <c r="L19" s="6" t="n">
@@ -1926,15 +1930,15 @@
         <v>45849.99930555555</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>GATT PERU S.R.L.; HERMES GROUP SAC</t>
-        </is>
-      </c>
-      <c r="P19" s="10" t="n">
-        <v>488990</v>
+          <t>GATT PERU S.R.L.</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="n">
+        <v>248990</v>
       </c>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="5" t="inlineStr">
@@ -1943,7 +1947,7 @@
         </is>
       </c>
       <c r="S19" s="6" t="n">
-        <v>45966.75679398148</v>
+        <v>45910.79685185185</v>
       </c>
       <c r="T19" s="5" t="inlineStr">
         <is>
@@ -1952,98 +1956,10 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 477 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 478 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
         </is>
       </c>
       <c r="V19" s="8" t="inlineStr">
-        <is>
-          <t>Ver proceso</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>1131459</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Concurso Público Abreviado</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>45846.64722222222</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>477</v>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="10" t="n">
-        <v>278000</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>45847.00069444445</v>
-      </c>
-      <c r="M20" s="6" t="n">
-        <v>45849.99930555555</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>GATT PERU S.R.L.</t>
-        </is>
-      </c>
-      <c r="P20" s="10" t="n">
-        <v>248990</v>
-      </c>
-      <c r="Q20" s="4" t="n"/>
-      <c r="R20" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
-        </is>
-      </c>
-      <c r="S20" s="6" t="n">
-        <v>45910.79685185185</v>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Retrotraído/reiniciado: revisar nueva etapa del cronograma.</t>
-        </is>
-      </c>
-      <c r="U20" s="5" t="inlineStr">
-        <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 477 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
-        </is>
-      </c>
-      <c r="V20" s="8" t="inlineStr">
         <is>
           <t>Ver proceso</t>
         </is>
@@ -2066,11 +1982,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2081,7 +1996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2157,7 +2072,7 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2193,7 +2108,7 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -2211,7 +2126,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -2221,15 +2136,15 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>PRESTACIONES PENDIENTES PARA LA EJECUCION DEL SALDO DE OBRA DEL PROYECTO CONSTRUCCIÓN Y ADECUACIÓN DE INFRAESTRUCTURA INTERNA, EXTERNA Y ZONAS DE INFLUENCIA DIRECTA DE LA CLÍNICA UNIVERSITARIA DENTRO DE LA UNMSM¿PRESTACIONES PENDIENTES PARA LA EJEC</t>
+          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>CONSENTIDO</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="n">
+          <t>CONVOCADO</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2237,19 +2152,17 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n">
-        <v>3829503.56</v>
-      </c>
+      <c r="G4" s="4" t="n"/>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE INFRAESTRUCTURA DE SALUD</t>
+          <t>RENOVACION DEL SOPORTE Y MANTENIMIENTO DE LICENCIAS DE SOFTWARE PARA EL ERP SAP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -2259,7 +2172,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE RENOVACIÓN DE SUSCRIPCION DE LICENCIA, AMPLIACION DE COBERTURA DE PROTECCION Y CAPACIDAD DE ALMACENAMIENTO EN NUBE, CAPACITACION Y SOPORTE TECNICO DE LA PLATAFORMA DE RESPALDO Y RESTAURACION ACRONIS CYBER PROTECT DE LA MARCA ACRONIS</t>
+          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2267,25 +2180,21 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>RENOVACION DEL SOPORTE Y MANTENIMIENTO DE LICENCIAS DE SOFTWARE PARA EL ERP SAP</t>
-        </is>
-      </c>
+      <c r="H5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2295,7 +2204,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGUROS PATRIMONIALES, MULTIRIESGO, 3D RESPONSABILIDAD CIVIL, VEHICULOS, ACCIDENTES PERSONALES, SEGURO DE VEHICULOS AEREO NO TRIPULADO Y SEGURO TREC</t>
+          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2303,21 +2212,25 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Servicio</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>SERVICIO DE CABLEADO ESTRUCTURADO Y CONEXION DE FIBRA OPTICA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2327,15 +2240,15 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE IMPLEMENTACIÓN INTEGRAL DE LA INFRAESTRUCTURA DE COMUNICACIONES (CABLEADO ESTRUCTURADO Y FIBRA ÓPTICA) DEL COSAC I</t>
+          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="n">
+          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -2343,17 +2256,19 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G7" s="4" t="n"/>
+      <c r="G7" s="9" t="n">
+        <v>481750</v>
+      </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE CABLEADO ESTRUCTURADO Y CONEXION DE FIBRA OPTICA</t>
+          <t>SERVICIO DE ALQUILER DE GRUA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2363,15 +2278,15 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de grúas para las acciones traslados internos de vehículos en depósito y el proceso de chatarreo de vehículos de la Dirección de Fiscalización y Sanción de la ATU</t>
+          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n">
+          <t>APELADO</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2379,37 +2294,37 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G8" s="10" t="n">
-        <v>481750</v>
+      <c r="G8" s="9" t="n">
+        <v>3565508.55</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE GRUA</t>
+          <t>SERVICIO DE ALQUILER DE VEHICULOS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE TRASLADO DE PERSONAL DE FISCALIZACION</t>
+          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 -CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>APELADO</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="n">
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -2417,50 +2332,48 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G9" s="10" t="n">
-        <v>3565508.55</v>
+      <c r="G9" s="9" t="n">
+        <v>4933726.01</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE VEHICULOS</t>
+          <t>CONSTRUCCION DE CARRETERA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>IOARR: ¿RENOVACION DE PARADEROS; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO Nº 2 -CORREDOR ROJO CON RECORRIDO EN LOS PRINCIPALES EJES VIALES DE LOS DISTRITOS; SAN MIGUEL, PUEBLO LIBRE, MAGDALENA DEL MAR, JESUS MARÍA, SAN ISIDRO, LINCE</t>
+          <t>BALDOSA PODOTACTIL DE GUIA</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>1</v>
+          <t>CONVOCADO_POR_REINICIO</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>8000</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>4933726.01</v>
-      </c>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE CARRETERA</t>
+          <t>PISO DE JEBE DE 4 mm X 0.40 m X 0.60 m</t>
         </is>
       </c>
     </row>
@@ -2472,12 +2385,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>BALDOSA PODOTACTIL DE GUIA</t>
+          <t>BALDOSA PODOTACTIL DE ALERTA</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -2485,8 +2398,8 @@
           <t>CONVOCADO_POR_REINICIO</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
-        <v>8000</v>
+      <c r="E11" s="9" t="n">
+        <v>3000</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
@@ -2503,7 +2416,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2513,33 +2426,33 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>BALDOSA PODOTACTIL DE ALERTA</t>
+          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO_POR_REINICIO</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>3000</v>
+          <t>CONVOCADO</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Servicio</t>
         </is>
       </c>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>PISO DE JEBE DE 4 mm X 0.40 m X 0.60 m</t>
+          <t>SERVICIO DE SEGURIDAD Y VIGILANCIA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -2549,7 +2462,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD PATRIMONIAL DE LA INFRAESTRUCTURA E INSTALACIÓN DEL CORREDOR SEGREGADO DE ALTA CAPACIDAD (COSAC) DE LA ATU</t>
+          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2557,7 +2470,7 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2568,14 +2481,14 @@
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE SEGURIDAD Y VIGILANCIA</t>
+          <t>SERVICIO DE MANTENIMIENTO DE PUERTAS LEVADIZAS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -2585,7 +2498,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO CORRECTIVO DE LAS PUERTAS AUTOMÁTICAS DE LA ESTACIÓN CENTRAL DEL COSAC I</t>
+          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RE</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2593,7 +2506,7 @@
           <t>CONVOCADO</t>
         </is>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -2604,14 +2517,14 @@
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE MANTENIMIENTO DE PUERTAS LEVADIZAS</t>
+          <t>CONSTRUCCION DE ESTACION PARA EMBARQUE DE PASAJEROS DE TRANSPORTE URBANO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -2621,33 +2534,35 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO PARA LA ELABORACION DEL EXPEDIENTE TECNICO Y EJECUCION DE LA OBRA POR MODALIDAD DE DISEÑO Y CONSTRUCCION DE LA FASE 1 DEL PROYECTO: RENOVACION DE PARADERO; EN EL SERVICIO DE TRANSPORTE DEL CORREDOR COMPLEMENTARIO N° 2 ¿ CORREDOR ROJO, CON RE</t>
+          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n">
+          <t>CONSENTIDO</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Servicio</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="n"/>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>395000</v>
+      </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCION DE ESTACION PARA EMBARQUE DE PASAJEROS DE TRANSPORTE URBANO</t>
+          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-1-2025-ATU-1</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2657,28 +2572,28 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>CONSENTIDO</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="n">
+          <t>RETROTRAIDO_POR_RESOLUCION</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>395000</v>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>278000</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN E INSTALACIÓN DE GRUPO ELECTRÓGENO INSONORO DE 250 KVA PARA LA SEDE DE LIMA DE LA AUTORIDAD DE TRANSPORTE URBANO PARA LIMA Y CALLAO</t>
+          <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2618,7 @@
           <t>RETROTRAIDO_POR_RESOLUCION</t>
         </is>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2711,48 +2626,10 @@
           <t>Servicio</t>
         </is>
       </c>
-      <c r="G17" s="10" t="n">
+      <c r="G17" s="9" t="n">
         <v>278000</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE ABASTECIMIENTO DE AGUA A TRAVÉS DE UN CAMIÓN CISTERNA PARA LA LIMPIEZA DE LAS ESTACIONES DEL COSAC</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>RETROTRAIDO_POR_RESOLUCION</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Servicio</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>278000</v>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>SERVICIO DE ABASTECIMIENTO DE AGUA POTABLE EN CAMIONES CISTERNA</t>
         </is>
@@ -2772,7 +2649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2862,11 +2739,11 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP SER-SM-7-2026-ATU-1</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>46304.93541666667</v>
+        <v>46296.87777777778</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -2887,11 +2764,11 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP SER-SM-6-2026-ATU-1</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>46307.87658564815</v>
+        <v>46276.85416666666</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -2900,7 +2777,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -2912,20 +2789,20 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>RES-PROC-3-2026-CD/SAPLI-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46307.87658564815</v>
+        <v>46224.80069444444</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -2937,20 +2814,20 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-7-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>46296.87777777778</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -2962,11 +2839,11 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-6-2026-ATU-1</t>
+          <t>CP SER-SM-2-2026-ATU-1</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>46276.85416666666</v>
+        <v>46318.75248842593</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -2975,7 +2852,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -2987,11 +2864,11 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>46224.80069444444</v>
+        <v>46217.80902777778</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -3012,11 +2889,11 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>46318.75248842593</v>
+        <v>46239.78258101852</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -3037,11 +2914,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-2-2026-ATU-1</t>
+          <t>CP-ABR-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>46318.75248842593</v>
+        <v>46239.78258101852</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -3066,7 +2943,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>46217.80902777778</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
@@ -3075,7 +2952,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -3091,16 +2968,16 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>46239.78258101852</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -3116,16 +2993,16 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>46239.78258101852</v>
+        <v>46247.7293287037</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3137,11 +3014,11 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46199.81041666667</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
@@ -3150,7 +3027,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -3162,20 +3039,20 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46217.74835648148</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -3187,20 +3064,20 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-5-2026-ATU-1</t>
+          <t>CP SER-SM-5-2026-ATU-1</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>46247.7293287037</v>
+        <v>46217.74835648148</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -3216,18 +3093,10 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>46199.81041666667</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Bases Administrativas</t>
-        </is>
-      </c>
+        <v>46268.96559027778</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3241,18 +3110,10 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>46217.74835648148</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Absolución de consultas</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
-        </is>
-      </c>
+        <v>46268.96734953704</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3266,7 +3127,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>46217.74835648148</v>
+        <v>46295.72564814815</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
@@ -3275,7 +3136,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -3291,10 +3152,18 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>46268.96559027778</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr"/>
+        <v>46295.72565972222</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Evaluación / cuadro comparativo</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Calificación y Evaluación</t>
+        </is>
+      </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3308,10 +3177,18 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>46268.96734953704</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
+        <v>46295.72565972222</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Buena pro</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
+        </is>
+      </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3321,11 +3198,11 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>46295.72564814815</v>
+        <v>46181.99722222222</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
@@ -3334,7 +3211,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3346,20 +3223,20 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46205.90194444444</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -3371,20 +3248,20 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-5-2026-ATU-1</t>
+          <t>LP-ABR-2-2026--ATU-1</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>46295.72565972222</v>
+        <v>46205.90195601852</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -3400,7 +3277,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>46181.99722222222</v>
+        <v>46226.00878472222</v>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
@@ -3409,7 +3286,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -3425,16 +3302,16 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>46205.90194444444</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -3450,16 +3327,16 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>46205.90195601852</v>
+        <v>46226.00881944445</v>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -3471,11 +3348,11 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>46226.00878472222</v>
+        <v>46013.78333333333</v>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
@@ -3484,7 +3361,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -3496,20 +3373,20 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46021.28239583333</v>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Acta de no formulación de consultas y observaciones</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -3521,20 +3398,20 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-2-2026--ATU-1</t>
+          <t>LP-ABR-7-2025-ATU-1</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>46226.00881944445</v>
+        <v>46021.70075231481</v>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -3550,7 +3427,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>46013.78333333333</v>
+        <v>46043.68869212963</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
@@ -3559,7 +3436,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -3575,16 +3452,16 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>46021.28239583333</v>
+        <v>46043.68869212963</v>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Acta de no formulación de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -3600,16 +3477,16 @@
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>46021.70075231481</v>
+        <v>46043.6887037037</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -3625,18 +3502,10 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>46043.68869212963</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Presentación de Propuestas</t>
-        </is>
-      </c>
+        <v>46077.64881944445</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3650,16 +3519,16 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>46043.68869212963</v>
+        <v>46077.65069444444</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -3675,7 +3544,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>46043.6887037037</v>
+        <v>46077.6509375</v>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
@@ -3700,10 +3569,18 @@
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>46077.64881944445</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="5" t="inlineStr"/>
+        <v>46077.65246527778</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Buena pro</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
+        </is>
+      </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -3717,7 +3594,7 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>46077.65069444444</v>
+        <v>46077.67525462963</v>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
@@ -3742,7 +3619,7 @@
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>46077.6509375</v>
+        <v>46077.67789351852</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
@@ -3767,7 +3644,7 @@
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>46077.65246527778</v>
+        <v>46077.67956018518</v>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
@@ -3792,7 +3669,7 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>46077.67525462963</v>
+        <v>46077.75027777778</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
@@ -3813,20 +3690,20 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>CP SER-SM-3-2025-ATU-1</t>
         </is>
       </c>
       <c r="B43" s="6" t="n">
-        <v>46077.67789351852</v>
+        <v>45958.84930555556</v>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -3838,20 +3715,20 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>CP-ABR-4-2025-ATU-2</t>
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>46077.67956018518</v>
+        <v>45936.61597222222</v>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -3863,20 +3740,20 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-7-2025-ATU-1</t>
+          <t>LP-ABR-6-2025-ATU-1</t>
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>46077.75027777778</v>
+        <v>45936.87291666667</v>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -3888,11 +3765,11 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>CP SER-SM-3-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>45958.84930555556</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
@@ -3913,11 +3790,11 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>CP-ABR-4-2025-ATU-2</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>45936.61597222222</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
@@ -3926,7 +3803,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Resumen ejecutivo</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -3938,20 +3815,20 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>LP-ABR-6-2025-ATU-1</t>
+          <t>AS-SM-15-2024-ATU-4</t>
         </is>
       </c>
       <c r="B48" s="6" t="n">
-        <v>45936.87291666667</v>
+        <v>45931.69513888889</v>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Informe que sustenta la declaratoria de Desierto</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -3967,16 +3844,16 @@
         </is>
       </c>
       <c r="B49" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45945.71658564815</v>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -3992,7 +3869,7 @@
         </is>
       </c>
       <c r="B50" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45945.71658564815</v>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
@@ -4001,7 +3878,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Resumen ejecutivo</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -4017,16 +3894,16 @@
         </is>
       </c>
       <c r="B51" s="6" t="n">
-        <v>45931.69513888889</v>
+        <v>45953.42690972222</v>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Informe que sustenta la declaratoria de Desierto</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -4042,16 +3919,16 @@
         </is>
       </c>
       <c r="B52" s="6" t="n">
-        <v>45945.71658564815</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -4067,16 +3944,16 @@
         </is>
       </c>
       <c r="B53" s="6" t="n">
-        <v>45945.71658564815</v>
+        <v>45953.4269212963</v>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -4088,11 +3965,11 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-1-2025-ATU-1</t>
         </is>
       </c>
       <c r="B54" s="6" t="n">
-        <v>45953.42690972222</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
@@ -4101,7 +3978,7 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Presentación de Propuestas</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -4113,20 +3990,20 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-1-2025-ATU-1</t>
         </is>
       </c>
       <c r="B55" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45902.81356481482</v>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Absolución de consultas</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Pliego de absolución de consultas y observaciones</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -4138,20 +4015,20 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>AS-SM-15-2024-ATU-4</t>
+          <t>CP-ABR-1-2025-ATU-1</t>
         </is>
       </c>
       <c r="B56" s="6" t="n">
-        <v>45953.4269212963</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -4167,7 +4044,7 @@
         </is>
       </c>
       <c r="B57" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45910.79684027778</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
@@ -4176,7 +4053,7 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -4192,16 +4069,16 @@
         </is>
       </c>
       <c r="B58" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45937.76886574074</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -4217,16 +4094,16 @@
         </is>
       </c>
       <c r="B59" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45937.76886574074</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -4242,18 +4119,10 @@
         </is>
       </c>
       <c r="B60" s="6" t="n">
-        <v>45910.79684027778</v>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Presentación de Propuestas</t>
-        </is>
-      </c>
+        <v>45966.75502314815</v>
+      </c>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr"/>
       <c r="E60" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4267,16 +4136,16 @@
         </is>
       </c>
       <c r="B61" s="6" t="n">
-        <v>45937.76886574074</v>
+        <v>45966.75679398148</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Evaluación / cuadro comparativo</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Calificación y Evaluación</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -4292,16 +4161,16 @@
         </is>
       </c>
       <c r="B62" s="6" t="n">
-        <v>45937.76886574074</v>
+        <v>45846.64722222222</v>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Administrativas</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -4317,10 +4186,18 @@
         </is>
       </c>
       <c r="B63" s="6" t="n">
-        <v>45966.75502314815</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr"/>
-      <c r="D63" s="5" t="inlineStr"/>
+        <v>45902.81356481482</v>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Absolución de consultas</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Pliego de absolución de consultas y observaciones</t>
+        </is>
+      </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
@@ -4334,16 +4211,16 @@
         </is>
       </c>
       <c r="B64" s="6" t="n">
-        <v>45966.75679398148</v>
+        <v>45902.81357638889</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Buena pro</t>
+          <t>Bases</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
+          <t>Bases Integradas</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -4359,7 +4236,7 @@
         </is>
       </c>
       <c r="B65" s="6" t="n">
-        <v>45846.64722222222</v>
+        <v>45910.79684027778</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
@@ -4368,7 +4245,7 @@
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Bases Administrativas</t>
+          <t>Documentos de Presentación de Propuestas</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -4384,16 +4261,16 @@
         </is>
       </c>
       <c r="B66" s="6" t="n">
-        <v>45902.81356481482</v>
+        <v>45910.79685185185</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Absolución de consultas</t>
+          <t>Evaluación / cuadro comparativo</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Pliego de absolución de consultas y observaciones</t>
+          <t>Documentos de Calificación y Evaluación</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -4409,94 +4286,19 @@
         </is>
       </c>
       <c r="B67" s="6" t="n">
-        <v>45902.81357638889</v>
+        <v>45910.79685185185</v>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Bases</t>
+          <t>Buena pro</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Bases Integradas</t>
+          <t>Documentos de Otorgamiento de Buena Pro</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
-        </is>
-      </c>
-      <c r="B68" s="6" t="n">
-        <v>45910.79684027778</v>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Bases</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Presentación de Propuestas</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="n">
-        <v>45910.79685185185</v>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Evaluación / cuadro comparativo</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Calificación y Evaluación</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>CP-ABR-1-2025-ATU-1</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="n">
-        <v>45910.79685185185</v>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Buena pro</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Documentos de Otorgamiento de Buena Pro</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4570,13 +4372,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4629,17 +4428,17 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONSENTIDO</t>
+          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>PENDIENTE_DE_REGISTRO_DE_EFECTO</t>
+          <t>APELADO</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -4649,7 +4448,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>APELADO</t>
+          <t>CONVOCADO_POR_REINICIO</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -4659,7 +4458,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CONVOCADO_POR_REINICIO</t>
+          <t>CONSENTIDO</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">

</xml_diff>

<commit_message>
Actualiza procesos SEACE (30/10/2026 08:41)
</commit_message>
<xml_diff>
--- a/seace/Procesos_SEACE_ATU.xlsx
+++ b/seace/Procesos_SEACE_ATU.xlsx
@@ -617,7 +617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Convocatorias desde 2025 · Revisados: 102 · Vigentes: 15 · Generado: 29/10/2026 08:30 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
+          <t>Convocatorias desde 2025 · Revisados: 102 · Vigentes: 15 · Generado: 30/10/2026 08:41 · Fuente: OECE – Contrataciones Abiertas (datos SEACE)</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         <v>46321.88611111111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -797,12 +797,12 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Consultas y observaciones hasta el 29/10/2026 (vence hoy).</t>
+          <t>Convocado: etapa de consultas cerrada; en curso hacia presentación de ofertas/evaluación.</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 26/10/2026 (hace 3 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (26/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 26/10/2026 (hace 4 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (26/10/2026).</t>
         </is>
       </c>
       <c r="V5" s="8" t="inlineStr">
@@ -844,7 +844,7 @@
         <v>46317.78611111111</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 7 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 22/10/2026 (hace 8 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (22/10/2026).</t>
         </is>
       </c>
       <c r="V6" s="8" t="inlineStr">
@@ -922,7 +922,7 @@
         <v>46296.87777777778</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 28 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 01/10/2026 (hace 29 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (01/10/2026).</t>
         </is>
       </c>
       <c r="V7" s="8" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v>46276.85416666666</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 48 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 11/09/2026 (hace 49 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (11/09/2026).</t>
         </is>
       </c>
       <c r="V8" s="8" t="inlineStr">
@@ -1078,7 +1078,7 @@
         <v>46224.80069444444</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 100 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
+          <t>Concurso Público de Servicios convocado el 21/07/2026 (hace 101 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Integradas (23/10/2026).</t>
         </is>
       </c>
       <c r="V9" s="8" t="inlineStr">
@@ -1156,7 +1156,7 @@
         <v>46217.80902777778</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 107 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 14/07/2026 (hace 108 días). Valor estimado/referencial: S/ 481,750.00. Estado: PENDIENTE_DE_REGISTRO_DE_EFECTO. Postores: 10. Buena pro a LOGISTAS SERVICIOS S.A.C. por S/ 315,952.00. Último documento: Documentos de Otorgamiento de Buena Pro (13/08/2026).</t>
         </is>
       </c>
       <c r="V10" s="8" t="inlineStr">
@@ -1244,7 +1244,7 @@
         <v>46199.81041666667</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 125 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
+          <t>Concurso Público de Servicios convocado el 26/06/2026 (hace 126 días). Valor estimado/referencial: S/ 3,565,508.55. Estado: APELADO. Postores: 15. Último documento: Documentos de Otorgamiento de Buena Pro (30/09/2026).</t>
         </is>
       </c>
       <c r="V11" s="8" t="inlineStr">
@@ -1326,7 +1326,7 @@
         <v>46181.99722222222</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 143 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 08/06/2026 (hace 144 días). Valor estimado/referencial: S/ 4,933,726.01. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 64. Buena pro a CONSORCIO PROGRESO por S/ 4,687,039.71. Último documento: Documentos de Otorgamiento de Buena Pro (23/07/2026).</t>
         </is>
       </c>
       <c r="V12" s="8" t="inlineStr">
@@ -1414,7 +1414,7 @@
         <v>46013.78333333333</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 311 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
+          <t>Licitación Pública Abreviada de bienes convocado el 22/12/2025 (hace 312 días). Valor estimado/referencial: no publicado. 2 ítems: 2 CONVOCADO_POR_REINICIO. Postores: 17. Buena pro a SOLUCIONES ESPECIALES S.A.C. por S/ 468,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (24/02/2026).</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -1500,7 +1500,7 @@
         <v>45958.84930555556</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 366 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 367 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 366 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
+          <t>Concurso Público de Servicios convocado el 28/10/2025 (hace 367 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (28/10/2025).</t>
         </is>
       </c>
       <c r="V14" s="8" t="inlineStr">
@@ -1578,7 +1578,7 @@
         <v>45936.61597222222</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1609,12 +1609,12 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 388 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 389 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 388 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 06/10/2025 (hace 389 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V15" s="8" t="inlineStr">
@@ -1656,7 +1656,7 @@
         <v>45936.87291666667</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Convocado sin documentos nuevos hace 388 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
+          <t>Convocado sin documentos nuevos hace 389 días: verificar en SEACE si sigue en curso o no fue actualizado.</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 388 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
+          <t>Licitación Pública Abreviada de obras convocado el 06/10/2025 (hace 389 días). Valor estimado/referencial: no publicado. Estado: CONVOCADO. Último documento: Bases Administrativas (06/10/2025).</t>
         </is>
       </c>
       <c r="V16" s="8" t="inlineStr">
@@ -1734,7 +1734,7 @@
         <v>45931.69513888889</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 393 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
+          <t>Adjudicación Simplificada de bienes convocado el 01/10/2025 (hace 394 días). Valor estimado/referencial: S/ 395,000.00. Estado: CONSENTIDO. Postores: 7. Buena pro a SERVFAC PERU E.I.R.L. por S/ 378,900.00. Último documento: Documentos de Otorgamiento de Buena Pro (23/10/2025).</t>
         </is>
       </c>
       <c r="V17" s="8" t="inlineStr">
@@ -1822,7 +1822,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 478 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 479 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 23. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Buena pro a HERMES GROUP SAC por S/ 240,000.00. Último documento: Documentos de Otorgamiento de Buena Pro (05/11/2025).</t>
         </is>
       </c>
       <c r="V18" s="8" t="inlineStr">
@@ -1910,7 +1910,7 @@
         <v>45846.64722222222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 478 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
+          <t>Concurso Público Abreviado de servicios convocado el 08/07/2025 (hace 479 días). Valor estimado/referencial: S/ 278,000.00. Estado: RETROTRAIDO_POR_RESOLUCION. Postores: 22. Buena pro a GATT PERU S.R.L. por S/ 248,990.00. Último documento: Documentos de Otorgamiento de Buena Pro (10/09/2025).</t>
         </is>
       </c>
       <c r="V19" s="8" t="inlineStr">

</xml_diff>